<commit_message>
Actualizar Junta Carter De Distribucion a categoria Distribucion
Motor > Distribución > Kits de Tapa de Distribución.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENbDrNFvGQL8kZiZLMZ8xH
</commit_message>
<xml_diff>
--- a/Inventario_Curado_Categorizado.xlsx
+++ b/Inventario_Curado_Categorizado.xlsx
@@ -13811,7 +13811,12 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Juntas, Sellos y Herrajes</t>
+          <t>Distribución</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Kits de Tapa de Distribución</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar Categoria5_ML para Juntas, Sellos y Herrajes
Juntas y Sellos / Kits de Herrajes según tipo de producto.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENbDrNFvGQL8kZiZLMZ8xH
</commit_message>
<xml_diff>
--- a/Inventario_Curado_Categorizado.xlsx
+++ b/Inventario_Curado_Categorizado.xlsx
@@ -580,6 +580,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -912,6 +917,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -957,6 +967,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1002,6 +1017,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1047,6 +1067,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1088,6 +1113,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1133,6 +1163,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1174,6 +1209,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1219,6 +1259,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1264,6 +1309,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1309,6 +1359,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1354,6 +1409,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1399,6 +1459,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1444,6 +1509,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1489,6 +1559,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1534,6 +1609,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1579,6 +1659,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1624,6 +1709,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1669,6 +1759,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1714,6 +1809,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1759,6 +1859,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1804,6 +1909,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1849,6 +1959,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1894,6 +2009,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1935,6 +2055,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1976,6 +2101,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2021,6 +2151,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2066,6 +2201,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2111,6 +2251,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2156,6 +2301,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2201,6 +2351,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2246,6 +2401,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2291,6 +2451,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2336,6 +2501,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2381,6 +2551,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2426,6 +2601,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2471,6 +2651,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2516,6 +2701,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2561,6 +2751,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2606,6 +2801,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -2651,6 +2851,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2696,6 +2901,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -2741,6 +2951,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2786,6 +3001,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -2827,6 +3047,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2872,6 +3097,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -2917,6 +3147,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2962,6 +3197,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -3007,6 +3247,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3052,6 +3297,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -3097,6 +3347,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3142,6 +3397,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -3187,6 +3447,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3232,6 +3497,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -3277,6 +3547,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3322,6 +3597,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -3367,6 +3647,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3412,6 +3697,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4097,6 +4387,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4138,6 +4433,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -4179,6 +4479,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4220,6 +4525,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -4261,6 +4571,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4302,6 +4617,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -4343,6 +4663,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4384,6 +4709,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -4425,6 +4755,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4466,6 +4801,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -4507,6 +4847,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4548,6 +4893,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -4589,6 +4939,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4630,6 +4985,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -4671,6 +5031,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4712,6 +5077,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -4757,6 +5127,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4802,6 +5177,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -4847,6 +5227,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4892,6 +5277,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -4937,6 +5327,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4978,6 +5373,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -5019,6 +5419,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5064,6 +5469,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -5109,6 +5519,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5154,6 +5569,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -5199,6 +5619,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5244,6 +5669,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -5289,6 +5719,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5334,6 +5769,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -5379,6 +5819,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5424,6 +5869,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -5465,6 +5915,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5510,6 +5965,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -5555,6 +6015,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5596,6 +6061,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -5641,6 +6111,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5686,6 +6161,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -5731,6 +6211,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -5772,6 +6257,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -5817,6 +6307,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -5862,6 +6357,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -5907,6 +6407,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -5952,6 +6457,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -5997,6 +6507,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6042,6 +6557,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -6087,6 +6607,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6132,6 +6657,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -6177,6 +6707,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6222,6 +6757,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -6267,6 +6807,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -6312,6 +6857,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -6357,6 +6907,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6402,6 +6957,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -6447,6 +7007,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -6492,6 +7057,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -6537,6 +7107,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -6582,6 +7157,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -6627,6 +7207,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -6672,6 +7257,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -6717,6 +7307,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -6762,6 +7357,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -6807,6 +7407,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6852,6 +7457,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -6891,6 +7501,11 @@
       <c r="I147" t="inlineStr">
         <is>
           <t>Juntas, Sellos y Herrajes</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
         </is>
       </c>
     </row>
@@ -10410,6 +11025,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -10455,6 +11075,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -10500,6 +11125,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -10545,6 +11175,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -10590,6 +11225,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -10635,6 +11275,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -10676,6 +11321,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -10721,6 +11371,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -10766,6 +11421,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -10811,6 +11471,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -10856,6 +11521,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -10901,6 +11571,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -10946,6 +11621,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -10991,6 +11671,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -11036,6 +11721,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -11081,6 +11771,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -11126,6 +11821,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -11171,6 +11871,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -11216,6 +11921,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -11261,6 +11971,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -11306,6 +12021,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -11351,6 +12071,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -11396,6 +12121,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -11441,6 +12171,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -11486,6 +12221,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -11531,6 +12271,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -11576,6 +12321,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -11621,6 +12371,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11666,6 +12421,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -11711,6 +12471,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11756,6 +12521,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -11801,6 +12571,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11846,6 +12621,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -11891,6 +12671,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11936,6 +12721,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -11981,6 +12771,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12026,6 +12821,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -12071,6 +12871,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Kits de Herrajes</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12112,6 +12917,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -12153,6 +12963,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12194,6 +13009,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -12235,6 +13055,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12280,6 +13105,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -12321,6 +13151,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12362,6 +13197,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -12403,6 +13243,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -12444,6 +13289,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -12489,6 +13339,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12530,6 +13385,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -12571,6 +13431,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12612,6 +13477,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -12653,6 +13523,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -12694,6 +13569,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -12735,6 +13615,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -12776,6 +13661,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -12817,6 +13707,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -12858,6 +13753,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -12903,6 +13803,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -12948,6 +13853,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -12989,6 +13899,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -13034,6 +13949,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -13079,6 +13999,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -13120,6 +14045,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -13161,6 +14091,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -13202,6 +14137,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -13243,6 +14183,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -13288,6 +14233,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -13413,6 +14363,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -13458,6 +14413,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -13503,6 +14463,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -13548,6 +14513,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -13593,6 +14563,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -13638,6 +14613,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -13683,6 +14663,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -13728,6 +14713,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -13771,6 +14761,11 @@
       <c r="I79" t="inlineStr">
         <is>
           <t>Juntas, Sellos y Herrajes</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
         </is>
       </c>
     </row>
@@ -13864,6 +14859,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -13909,6 +14909,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -13954,6 +14959,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -13999,6 +15009,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -14044,6 +15059,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -14089,6 +15109,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -14134,6 +15159,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -14179,6 +15209,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -14224,6 +15259,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -14269,6 +15309,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -14314,6 +15359,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -14359,6 +15409,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -14404,6 +15459,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -14449,6 +15509,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -14494,6 +15559,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -14539,6 +15609,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -14584,6 +15659,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -14629,6 +15709,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -14674,6 +15759,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -14719,6 +15809,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -14764,6 +15859,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -14809,6 +15909,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -14854,6 +15959,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -14899,6 +16009,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -14944,6 +16059,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -14989,6 +16109,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -15034,6 +16159,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -15079,6 +16209,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -15124,6 +16259,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -15169,6 +16309,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -15214,6 +16359,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -15259,6 +16409,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -15304,6 +16459,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -15349,6 +16509,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -15394,6 +16559,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -15439,6 +16609,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -15484,6 +16659,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -15529,6 +16709,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -16654,6 +17839,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -16699,6 +17889,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -16744,6 +17939,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -16789,6 +17989,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -16834,6 +18039,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -16879,6 +18089,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -16924,6 +18139,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -16969,6 +18189,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -17014,6 +18239,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
@@ -17059,6 +18289,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -17104,6 +18339,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -17149,6 +18389,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -17194,6 +18439,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -17239,6 +18489,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -17284,6 +18539,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -17329,6 +18589,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -17374,6 +18639,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -17419,6 +18689,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -17464,6 +18739,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -17509,6 +18789,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -17554,6 +18839,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -17599,6 +18889,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -17644,6 +18939,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -17689,6 +18989,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -17734,6 +19039,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -17779,6 +19089,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -17824,6 +19139,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -17869,6 +19189,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -17914,6 +19239,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -17959,6 +19289,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -18004,6 +19339,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -18049,6 +19389,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -18094,6 +19439,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -18139,6 +19489,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -18184,6 +19539,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -18229,6 +19589,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -18274,6 +19639,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -18319,6 +19689,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -18364,6 +19739,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -18409,6 +19789,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -18454,6 +19839,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -18499,6 +19889,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -18544,6 +19939,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
@@ -18585,6 +19985,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -18626,6 +20031,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
@@ -18667,6 +20077,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -18712,6 +20127,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
@@ -18757,6 +20177,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -18802,6 +20227,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -18847,6 +20277,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -18892,6 +20327,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
@@ -18937,6 +20377,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -18982,6 +20427,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
@@ -19027,6 +20477,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -19072,6 +20527,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
@@ -19117,6 +20577,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -19162,6 +20627,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -19207,6 +20677,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -19252,6 +20727,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
@@ -19293,6 +20773,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -19334,6 +20819,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -19375,6 +20865,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -19420,6 +20915,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
@@ -19465,6 +20965,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -19510,6 +21015,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
@@ -19555,6 +21065,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -19600,6 +21115,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
@@ -19645,6 +21165,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -19690,6 +21215,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
@@ -19735,6 +21265,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -19780,6 +21315,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
@@ -19825,6 +21365,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -19870,6 +21415,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
@@ -19915,6 +21465,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -19960,6 +21515,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
@@ -20005,6 +21565,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -20050,6 +21615,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
@@ -20095,6 +21665,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -20140,6 +21715,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="3" t="inlineStr">
@@ -20185,6 +21765,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -20230,6 +21815,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="3" t="inlineStr">
@@ -20275,6 +21865,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -20320,6 +21915,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
@@ -20365,6 +21965,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -20410,6 +22015,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="3" t="inlineStr">
@@ -20451,6 +22061,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -20496,6 +22111,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="3" t="inlineStr">
@@ -20541,6 +22161,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -20586,6 +22211,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="3" t="inlineStr">
@@ -20631,6 +22261,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -20676,6 +22311,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
@@ -20721,6 +22361,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -20766,6 +22411,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="3" t="inlineStr">
@@ -20811,6 +22461,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -20856,6 +22511,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
@@ -20901,6 +22561,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -20946,6 +22611,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
@@ -20991,6 +22661,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -21036,6 +22711,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="3" t="inlineStr">
@@ -21081,6 +22761,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -21126,6 +22811,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
@@ -21171,6 +22861,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -21216,6 +22911,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="3" t="inlineStr">
@@ -21261,6 +22961,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -21306,6 +23011,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="3" t="inlineStr">
@@ -21347,6 +23057,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -21392,6 +23107,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="3" t="inlineStr">
@@ -21437,6 +23157,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -21482,6 +23207,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="3" t="inlineStr">
@@ -21527,6 +23257,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -21572,6 +23307,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="3" t="inlineStr">
@@ -21617,6 +23357,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -21658,6 +23403,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="inlineStr">
@@ -21703,6 +23453,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -21748,6 +23503,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="3" t="inlineStr">
@@ -21793,6 +23553,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -21838,6 +23603,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="3" t="inlineStr">
@@ -21883,6 +23653,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -21928,6 +23703,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="inlineStr">
@@ -21973,6 +23753,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -22018,6 +23803,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
@@ -22063,6 +23853,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -22108,6 +23903,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="3" t="inlineStr">
@@ -22153,6 +23953,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -22198,6 +24003,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="3" t="inlineStr">
@@ -22243,6 +24053,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -22288,6 +24103,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="3" t="inlineStr">
@@ -22333,6 +24153,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -22378,6 +24203,11 @@
           <t>Juntas, Sellos y Herrajes</t>
         </is>
       </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="3" t="inlineStr">
@@ -22421,6 +24251,11 @@
       <c r="I275" t="inlineStr">
         <is>
           <t>Juntas, Sellos y Herrajes</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Juntas y Sellos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar Categoria6_ML para Juntas y Sellos
Clasificacion detallada: Juntas de Tapa de Cilindro, Admision,
Tapa de Valvulas, Carter, Kits de Juntas, Sellos de Admision, etc.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENbDrNFvGQL8kZiZLMZ8xH
</commit_message>
<xml_diff>
--- a/Inventario_Curado_Categorizado.xlsx
+++ b/Inventario_Curado_Categorizado.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:K169"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="26" defaultRowHeight="15"/>
   <cols>
     <col width="96.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -539,6 +539,11 @@
           <t>Categoria5_ML</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Categoria6_ML</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -585,6 +590,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1964,6 +1974,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2014,6 +2029,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2060,6 +2080,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2106,6 +2131,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2156,6 +2186,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2206,6 +2241,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2256,6 +2296,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2306,6 +2351,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2356,6 +2406,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Juntas de Motor</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2406,6 +2461,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Juntas de Motor</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2456,6 +2516,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2506,6 +2571,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2556,6 +2626,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2606,6 +2681,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2656,6 +2736,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2706,6 +2791,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2756,6 +2846,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2806,6 +2901,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -2856,6 +2956,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2906,6 +3011,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -2956,6 +3066,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3006,6 +3121,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -3052,6 +3172,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3102,6 +3227,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -3152,6 +3282,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3202,6 +3337,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -3252,6 +3392,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3302,6 +3447,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -3352,6 +3502,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3402,6 +3557,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -3452,6 +3612,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3502,6 +3667,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -3552,6 +3722,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3602,6 +3777,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -3652,6 +3832,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3702,6 +3887,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4392,6 +4582,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4438,6 +4633,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -4484,6 +4684,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4530,6 +4735,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -4576,6 +4786,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4622,6 +4837,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -4668,6 +4888,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4714,6 +4939,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -4760,6 +4990,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4806,6 +5041,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -4852,6 +5092,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4898,6 +5143,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -4944,6 +5194,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4990,6 +5245,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -5036,6 +5296,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5082,6 +5347,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -5132,6 +5402,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5182,6 +5457,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -5232,6 +5512,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5282,6 +5567,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -5332,6 +5622,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5378,6 +5673,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -5424,6 +5724,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5474,6 +5779,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -5524,6 +5834,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5574,6 +5889,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -5624,6 +5944,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5674,6 +5999,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -5724,6 +6054,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5774,6 +6109,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -5824,6 +6164,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5874,6 +6219,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -5920,6 +6270,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5970,6 +6325,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -6020,6 +6380,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6066,6 +6431,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -6116,6 +6486,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6166,6 +6541,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -6216,6 +6596,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6262,6 +6647,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -6312,6 +6702,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6362,6 +6757,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -6412,6 +6812,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6462,6 +6867,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -6512,6 +6922,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6562,6 +6977,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -6612,6 +7032,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6662,6 +7087,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -6712,6 +7142,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6762,6 +7197,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -6812,6 +7252,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -6862,6 +7307,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -6912,6 +7362,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6962,6 +7417,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -7012,6 +7472,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -7062,6 +7527,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -7112,6 +7582,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -7162,6 +7637,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -7212,6 +7692,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -7262,6 +7747,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -7312,6 +7802,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -7362,6 +7857,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -7412,6 +7912,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -7462,6 +7967,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -7506,6 +8016,11 @@
       <c r="J147" t="inlineStr">
         <is>
           <t>Juntas y Sellos</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Sellos de Admisión</t>
         </is>
       </c>
     </row>
@@ -8507,7 +9022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="38.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8571,6 +9086,11 @@
           <t>Categoria5_ML</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Categoria6_ML</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -10924,7 +11444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J323"/>
+  <dimension ref="A1:K323"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="140" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -10988,6 +11508,11 @@
           <t>Categoria5_ML</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Categoria6_ML</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -11030,6 +11555,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -12922,6 +13452,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -12968,6 +13503,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13014,6 +13554,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -13060,6 +13605,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13110,6 +13660,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -13156,6 +13711,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13202,6 +13762,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -13248,6 +13813,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13294,6 +13864,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -13344,6 +13919,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13390,6 +13970,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -13436,6 +14021,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13482,6 +14072,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -13528,6 +14123,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13574,6 +14174,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -13620,6 +14225,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13666,6 +14276,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -13712,6 +14327,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -13758,6 +14378,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -13808,6 +14433,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -13858,6 +14488,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -13904,6 +14539,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -13954,6 +14594,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -14004,6 +14649,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -14050,6 +14700,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -14096,6 +14751,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -14142,6 +14802,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -14188,6 +14853,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -14238,6 +14908,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Kits de Juntas</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -14368,6 +15043,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -14418,6 +15098,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -14468,6 +15153,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -14518,6 +15208,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -14568,6 +15263,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -14618,6 +15318,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -14668,6 +15373,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -14718,6 +15428,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -14766,6 +15481,11 @@
       <c r="J79" t="inlineStr">
         <is>
           <t>Juntas y Sellos</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Juntas de Cárter</t>
         </is>
       </c>
     </row>
@@ -14864,6 +15584,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -14914,6 +15639,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -14964,6 +15694,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -15014,6 +15749,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -15064,6 +15804,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -15114,6 +15859,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -15164,6 +15914,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -15214,6 +15969,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -15264,6 +16024,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -15314,6 +16079,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -15364,6 +16134,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -15414,6 +16189,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -15464,6 +16244,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -15514,6 +16299,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -15564,6 +16354,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -15614,6 +16409,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -15664,6 +16464,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -15714,6 +16519,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -15764,6 +16574,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -15814,6 +16629,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -15864,6 +16684,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -15914,6 +16739,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -15964,6 +16794,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -16014,6 +16849,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -16064,6 +16904,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -16114,6 +16959,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -16164,6 +17014,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -16214,6 +17069,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -16264,6 +17124,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -16314,6 +17179,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -16364,6 +17234,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -16414,6 +17289,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -16464,6 +17344,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -16514,6 +17399,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -16564,6 +17454,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -16614,6 +17509,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Juntas de Admisión</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -17844,6 +18744,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -17894,6 +18799,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -17944,6 +18854,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -17994,6 +18909,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -18044,6 +18964,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -18094,6 +19019,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -18144,6 +19074,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -18194,6 +19129,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -18244,6 +19184,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
@@ -18294,6 +19239,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -18344,6 +19294,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -18394,6 +19349,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -18444,6 +19404,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -18494,6 +19459,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -18544,6 +19514,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -18594,6 +19569,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -18644,6 +19624,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -18694,6 +19679,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -18744,6 +19734,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -18794,6 +19789,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -18844,6 +19844,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -18894,6 +19899,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -18944,6 +19954,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -18994,6 +20009,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -19044,6 +20064,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -19094,6 +20119,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -19144,6 +20174,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -19194,6 +20229,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -19244,6 +20284,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -19294,6 +20339,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -19344,6 +20394,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -19394,6 +20449,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -19444,6 +20504,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -19494,6 +20559,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -19544,6 +20614,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -19594,6 +20669,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -19644,6 +20724,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -19694,6 +20779,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -19744,6 +20834,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -19794,6 +20889,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -19844,6 +20944,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -19894,6 +20999,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -19944,6 +21054,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
@@ -19990,6 +21105,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -20036,6 +21156,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
@@ -20082,6 +21207,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -20132,6 +21262,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
@@ -20182,6 +21317,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -20232,6 +21372,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -20282,6 +21427,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -20332,6 +21482,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
@@ -20382,6 +21537,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -20432,6 +21592,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
@@ -20482,6 +21647,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -20532,6 +21702,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
@@ -20582,6 +21757,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -20632,6 +21812,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -20682,6 +21867,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -20732,6 +21922,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
@@ -20778,6 +21973,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -20824,6 +22024,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -20870,6 +22075,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -20920,6 +22130,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
@@ -20970,6 +22185,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -21020,6 +22240,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
@@ -21070,6 +22295,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -21120,6 +22350,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
@@ -21170,6 +22405,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -21220,6 +22460,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
@@ -21270,6 +22515,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -21320,6 +22570,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
@@ -21370,6 +22625,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -21420,6 +22680,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
@@ -21470,6 +22735,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -21520,6 +22790,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
@@ -21570,6 +22845,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -21620,6 +22900,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
@@ -21670,6 +22955,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -21720,6 +23010,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="3" t="inlineStr">
@@ -21770,6 +23065,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -21820,6 +23120,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="3" t="inlineStr">
@@ -21870,6 +23175,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -21920,6 +23230,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
@@ -21970,6 +23285,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -22020,6 +23340,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="3" t="inlineStr">
@@ -22066,6 +23391,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -22116,6 +23446,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="3" t="inlineStr">
@@ -22166,6 +23501,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -22216,6 +23556,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="3" t="inlineStr">
@@ -22266,6 +23611,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -22316,6 +23666,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
@@ -22366,6 +23721,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -22416,6 +23776,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="3" t="inlineStr">
@@ -22466,6 +23831,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -22516,6 +23886,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
@@ -22566,6 +23941,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -22616,6 +23996,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
@@ -22666,6 +24051,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -22716,6 +24106,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Cilindro</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="3" t="inlineStr">
@@ -22766,6 +24161,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -22816,6 +24216,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
@@ -22866,6 +24271,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -22916,6 +24326,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="3" t="inlineStr">
@@ -22966,6 +24381,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -23016,6 +24436,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="3" t="inlineStr">
@@ -23062,6 +24487,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -23112,6 +24542,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="3" t="inlineStr">
@@ -23162,6 +24597,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -23212,6 +24652,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="3" t="inlineStr">
@@ -23262,6 +24707,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -23312,6 +24762,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="3" t="inlineStr">
@@ -23362,6 +24817,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -23408,6 +24868,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="inlineStr">
@@ -23458,6 +24923,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -23508,6 +24978,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="3" t="inlineStr">
@@ -23558,6 +25033,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -23608,6 +25088,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="3" t="inlineStr">
@@ -23658,6 +25143,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -23708,6 +25198,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="inlineStr">
@@ -23758,6 +25253,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -23808,6 +25308,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
@@ -23858,6 +25363,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -23908,6 +25418,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="3" t="inlineStr">
@@ -23958,6 +25473,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -24008,6 +25528,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="3" t="inlineStr">
@@ -24058,6 +25583,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -24108,6 +25638,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="3" t="inlineStr">
@@ -24158,6 +25693,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -24208,6 +25748,11 @@
           <t>Juntas y Sellos</t>
         </is>
       </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="3" t="inlineStr">
@@ -24256,6 +25801,11 @@
       <c r="J275" t="inlineStr">
         <is>
           <t>Juntas y Sellos</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>Juntas de Tapa de Válvulas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar Cat6 Kits de Tornillos de Culata para Juego De Bulones
58 productos de Elring y Victor Reinz clasificados en
Motor > Juntas, Sellos y Herrajes > Kits de Herrajes > Kits de Tornillos de Culata.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENbDrNFvGQL8kZiZLMZ8xH
</commit_message>
<xml_diff>
--- a/Inventario_Curado_Categorizado.xlsx
+++ b/Inventario_Curado_Categorizado.xlsx
@@ -932,6 +932,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -982,6 +987,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1032,6 +1042,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1082,6 +1097,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1128,6 +1148,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1178,6 +1203,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1224,6 +1254,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1274,6 +1309,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1324,6 +1364,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1374,6 +1419,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1424,6 +1474,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1474,6 +1529,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1524,6 +1584,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1574,6 +1639,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1624,6 +1694,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1674,6 +1749,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1724,6 +1804,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1774,6 +1859,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1824,6 +1914,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1874,6 +1969,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1922,6 +2022,11 @@
       <c r="J30" t="inlineStr">
         <is>
           <t>Kits de Herrajes</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
         </is>
       </c>
     </row>
@@ -11610,6 +11715,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -11660,6 +11770,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -11710,6 +11825,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -11760,6 +11880,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -11810,6 +11935,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -11856,6 +11986,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -11906,6 +12041,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -11956,6 +12096,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -12006,6 +12151,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -12056,6 +12206,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -12106,6 +12261,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -12156,6 +12316,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -12206,6 +12371,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -12256,6 +12426,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -12306,6 +12481,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -12356,6 +12536,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -12406,6 +12591,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -12456,6 +12646,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -12506,6 +12701,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -12556,6 +12756,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -12606,6 +12811,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -12656,6 +12866,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -12706,6 +12921,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -12756,6 +12976,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -12806,6 +13031,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -12856,6 +13086,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -12906,6 +13141,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -12956,6 +13196,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -13006,6 +13251,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -13056,6 +13306,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -13106,6 +13361,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -13156,6 +13416,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -13206,6 +13471,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13256,6 +13526,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -13306,6 +13581,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13356,6 +13636,11 @@
           <t>Kits de Herrajes</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -13404,6 +13689,11 @@
       <c r="J39" t="inlineStr">
         <is>
           <t>Kits de Herrajes</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Kits de Tornillos de Culata</t>
         </is>
       </c>
     </row>

</xml_diff>